<commit_message>
perubahan template import excel data karyawan
</commit_message>
<xml_diff>
--- a/public/templates/TEMPLATE_IMPORT_KARYAWAN_HO.xlsx
+++ b/public/templates/TEMPLATE_IMPORT_KARYAWAN_HO.xlsx
@@ -26,109 +26,109 @@
     <t>NAMA LENGKAP *</t>
   </si>
   <si>
+    <t>NO. KTP (NIK) *</t>
+  </si>
+  <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>NIK HO</t>
+  </si>
+  <si>
+    <t>NO. TELEPON</t>
+  </si>
+  <si>
+    <t>TEMPAT LAHIR</t>
+  </si>
+  <si>
+    <t>TANGGAL LAHIR</t>
+  </si>
+  <si>
+    <t>TANGGAL MASUK</t>
+  </si>
+  <si>
+    <t>JABATAN</t>
+  </si>
+  <si>
+    <t>ALAMAT</t>
+  </si>
+  <si>
+    <t>AGAMA</t>
+  </si>
+  <si>
+    <t>PTKP</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>STATUS KARYAWAN</t>
+  </si>
+  <si>
+    <t>NAMA (SESUAI KTP)</t>
+  </si>
+  <si>
+    <t>NO. KK</t>
+  </si>
+  <si>
+    <t>RT/RW</t>
+  </si>
+  <si>
+    <t>KELURAHAN</t>
+  </si>
+  <si>
+    <t>KECAMATAN</t>
+  </si>
+  <si>
+    <t>PROPINSI</t>
+  </si>
+  <si>
+    <t>NPWP</t>
+  </si>
+  <si>
+    <t>EMAIL</t>
+  </si>
+  <si>
+    <t>LOKASI KERJA</t>
+  </si>
+  <si>
+    <t>START PKWT</t>
+  </si>
+  <si>
+    <t>END PKWT</t>
+  </si>
+  <si>
+    <t>NO. KONTRAK</t>
+  </si>
+  <si>
+    <t>NO. REKENING</t>
+  </si>
+  <si>
     <t>Wajib. Nama sesuai KTP.</t>
   </si>
   <si>
-    <t>NO. KTP (NIK) *</t>
-  </si>
-  <si>
     <t>Wajib. 16 digit.</t>
   </si>
   <si>
-    <t>UNIT</t>
-  </si>
-  <si>
     <t>Isi: HO-1 atau HO-2.</t>
   </si>
   <si>
-    <t>NIK HO</t>
-  </si>
-  <si>
     <t>Opsional. Nomor induk karyawan HO.</t>
   </si>
   <si>
-    <t>NO. TELEPON</t>
-  </si>
-  <si>
     <t>Opsional.</t>
   </si>
   <si>
-    <t>TEMPAT LAHIR</t>
-  </si>
-  <si>
-    <t>TANGGAL LAHIR</t>
-  </si>
-  <si>
     <t>Format DD-MM-YYYY (ketik sebagai teks).</t>
   </si>
   <si>
-    <t>TANGGAL MASUK</t>
-  </si>
-  <si>
-    <t>JABATAN</t>
-  </si>
-  <si>
     <t>Opsional. Ketik manual.</t>
   </si>
   <si>
-    <t>ALAMAT</t>
-  </si>
-  <si>
-    <t>AGAMA</t>
-  </si>
-  <si>
-    <t>PTKP</t>
-  </si>
-  <si>
     <t>Opsional. Contoh: TK/0, K/1.</t>
   </si>
   <si>
-    <t>STATUS</t>
-  </si>
-  <si>
     <t>AKTIF atau NONAKTIF. Default AKTIF.</t>
-  </si>
-  <si>
-    <t>STATUS KARYAWAN</t>
-  </si>
-  <si>
-    <t>NAMA (SESUAI KTP)</t>
-  </si>
-  <si>
-    <t>NO. KK</t>
-  </si>
-  <si>
-    <t>RT/RW</t>
-  </si>
-  <si>
-    <t>KELURAHAN</t>
-  </si>
-  <si>
-    <t>KECAMATAN</t>
-  </si>
-  <si>
-    <t>PROPINSI</t>
-  </si>
-  <si>
-    <t>NPWP</t>
-  </si>
-  <si>
-    <t>EMAIL</t>
-  </si>
-  <si>
-    <t>LOKASI KERJA</t>
-  </si>
-  <si>
-    <t>START PKWT</t>
-  </si>
-  <si>
-    <t>END PKWT</t>
-  </si>
-  <si>
-    <t>NO. KONTRAK</t>
-  </si>
-  <si>
-    <t>NO. REKENING</t>
   </si>
 </sst>
 </file>
@@ -558,188 +558,301 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="F3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="H3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="J3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="M3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="P3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="R3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="S3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="T3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="V3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="W3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="X3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="Y3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="Z3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="AA3" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="S3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="U3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="X3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="AA3" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:27" customHeight="1" ht="24">
       <c r="A4" s="4" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="U4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="W4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="X4" s="4" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="Y4" s="4" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="Z4" s="4" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="AA4" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" customHeight="1" ht="16"/>
-    <row r="6" spans="1:27" customHeight="1" ht="16"/>
-    <row r="7" spans="1:27" customHeight="1" ht="16"/>
-    <row r="8" spans="1:27" customHeight="1" ht="16"/>
-    <row r="9" spans="1:27" customHeight="1" ht="16"/>
-    <row r="10" spans="1:27" customHeight="1" ht="16"/>
-    <row r="11" spans="1:27" customHeight="1" ht="16"/>
-    <row r="12" spans="1:27" customHeight="1" ht="16"/>
-    <row r="13" spans="1:27" customHeight="1" ht="16"/>
-    <row r="14" spans="1:27" customHeight="1" ht="16"/>
-    <row r="15" spans="1:27" customHeight="1" ht="16"/>
-    <row r="16" spans="1:27" customHeight="1" ht="16"/>
-    <row r="17" spans="1:27" customHeight="1" ht="16"/>
-    <row r="18" spans="1:27" customHeight="1" ht="16"/>
-    <row r="19" spans="1:27" customHeight="1" ht="16"/>
-    <row r="20" spans="1:27" customHeight="1" ht="16"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" customHeight="1" ht="16">
+      <c r="C5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5"/>
+      <c r="N5"/>
+    </row>
+    <row r="6" spans="1:27" customHeight="1" ht="16">
+      <c r="C6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6"/>
+      <c r="N6"/>
+    </row>
+    <row r="7" spans="1:27" customHeight="1" ht="16">
+      <c r="C7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7"/>
+      <c r="N7"/>
+    </row>
+    <row r="8" spans="1:27" customHeight="1" ht="16">
+      <c r="C8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8"/>
+    </row>
+    <row r="9" spans="1:27" customHeight="1" ht="16">
+      <c r="C9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9"/>
+      <c r="N9"/>
+    </row>
+    <row r="10" spans="1:27" customHeight="1" ht="16">
+      <c r="C10"/>
+      <c r="K10"/>
+      <c r="L10"/>
+      <c r="M10"/>
+      <c r="N10"/>
+    </row>
+    <row r="11" spans="1:27" customHeight="1" ht="16">
+      <c r="C11"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11"/>
+      <c r="N11"/>
+    </row>
+    <row r="12" spans="1:27" customHeight="1" ht="16">
+      <c r="C12"/>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12"/>
+      <c r="N12"/>
+    </row>
+    <row r="13" spans="1:27" customHeight="1" ht="16">
+      <c r="C13"/>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13"/>
+      <c r="N13"/>
+    </row>
+    <row r="14" spans="1:27" customHeight="1" ht="16">
+      <c r="C14"/>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14"/>
+      <c r="N14"/>
+    </row>
+    <row r="15" spans="1:27" customHeight="1" ht="16">
+      <c r="C15"/>
+      <c r="K15"/>
+      <c r="L15"/>
+      <c r="M15"/>
+      <c r="N15"/>
+    </row>
+    <row r="16" spans="1:27" customHeight="1" ht="16">
+      <c r="C16"/>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16"/>
+      <c r="N16"/>
+    </row>
+    <row r="17" spans="1:27" customHeight="1" ht="16">
+      <c r="C17"/>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17"/>
+    </row>
+    <row r="18" spans="1:27" customHeight="1" ht="16">
+      <c r="C18"/>
+      <c r="K18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18"/>
+    </row>
+    <row r="19" spans="1:27" customHeight="1" ht="16">
+      <c r="C19"/>
+      <c r="K19"/>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19"/>
+    </row>
+    <row r="20" spans="1:27" customHeight="1" ht="16">
+      <c r="C20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:AA1"/>
     <mergeCell ref="A2:AA2"/>
   </mergeCells>
+  <dataValidations count="5">
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Unit harus salah satu dari: HO-1, HO-2" promptTitle="Unit" prompt="Pilih salah satu dari daftar: HO-1, HO-2" sqref="C5:C20">
+      <formula1>"HO-1,HO-2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Agama harus salah satu dari: Islam, Kristen Protestan, Kristen Katolik, Hindu, Buddha, Konghucu" promptTitle="Agama" prompt="Pilih salah satu dari daftar: Islam, Kristen Protestan, Kristen Katolik, Hindu, Buddha, Konghucu" sqref="K5:K20">
+      <formula1>"Islam,Kristen Protestan,Kristen Katolik,Hindu,Buddha,Konghucu"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="PTKP harus salah satu dari: TK/0, TK/1, TK/2, TK/3, K/0, K/1, K/2, K/3" promptTitle="PTKP" prompt="Pilih salah satu dari daftar: TK/0, TK/1, TK/2, TK/3, K/0, K/1, K/2, K/3" sqref="L5:L20">
+      <formula1>"TK/0,TK/1,TK/2,TK/3,K/0,K/1,K/2,K/3"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Status harus salah satu dari: AKTIF, NONAKTIF" promptTitle="Status" prompt="Pilih salah satu dari daftar: AKTIF, NONAKTIF" sqref="M5:M20">
+      <formula1>"AKTIF,NONAKTIF"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Status Karyawan harus salah satu dari: PKWT, PKWTT" promptTitle="Status Karyawan" prompt="Pilih salah satu dari daftar: PKWT, PKWTT" sqref="N5:N20">
+      <formula1>"PKWT,PKWTT"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>

</xml_diff>